<commit_message>
Levadas Te, Le e Co isoladas com partituras; volta imagem antiga do Swing 1
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_019LzxMs5ajBcG9V1K2gEhWs
</commit_message>
<xml_diff>
--- a/app_estudo_havayanas_exp/www/ritmos.xlsx
+++ b/app_estudo_havayanas_exp/www/ritmos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8242b9476157fafd/Aplicativos_Shiny/projeto_havayanas/app_estudo_havayanas/www/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8242b9476157fafd/Aplicativos_Shiny/projeto_havayanas/app_estudo_havayanas_exp/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{399CEAB1-49B8-BF4A-B210-06DC92F2808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F6C3C7B-5BE5-3C4C-A0BE-51BACA327EC4}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{399CEAB1-49B8-BF4A-B210-06DC92F2808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0707329-01D4-3E4A-A76F-7B08206131B5}"/>
   <bookViews>
-    <workbookView xWindow="-8640" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="levadas" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">convencoes!$A$1:$F$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">levadas!$A$1:$E$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">levadas!$A$1:$E$156</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="154">
   <si>
     <t>Levada</t>
   </si>
@@ -485,6 +485,21 @@
   </si>
   <si>
     <t>Alvaro</t>
+  </si>
+  <si>
+    <t>Le</t>
+  </si>
+  <si>
+    <t>Co</t>
+  </si>
+  <si>
+    <t>-- -- -- co | -- -- -- co | -- -- -- co | -- -- -- co</t>
+  </si>
+  <si>
+    <t>Te</t>
+  </si>
+  <si>
+    <t>-- te -- --  | -- te -- -- | -- te -- -- | -- te -- --</t>
   </si>
 </sst>
 </file>
@@ -818,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -2819,8 +2834,260 @@
         <v>139</v>
       </c>
     </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
+        <v>149</v>
+      </c>
+      <c r="B139" t="s">
+        <v>11</v>
+      </c>
+      <c r="C139" t="s">
+        <v>132</v>
+      </c>
+      <c r="D139" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>149</v>
+      </c>
+      <c r="B140" t="s">
+        <v>7</v>
+      </c>
+      <c r="C140" t="s">
+        <v>132</v>
+      </c>
+      <c r="D140" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
+        <v>149</v>
+      </c>
+      <c r="B141" t="s">
+        <v>6</v>
+      </c>
+      <c r="C141" t="s">
+        <v>132</v>
+      </c>
+      <c r="D141" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
+        <v>149</v>
+      </c>
+      <c r="B142" t="s">
+        <v>14</v>
+      </c>
+      <c r="C142" t="s">
+        <v>132</v>
+      </c>
+      <c r="D142" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
+        <v>149</v>
+      </c>
+      <c r="B143" t="s">
+        <v>16</v>
+      </c>
+      <c r="C143" t="s">
+        <v>132</v>
+      </c>
+      <c r="D143" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>149</v>
+      </c>
+      <c r="B144" t="s">
+        <v>9</v>
+      </c>
+      <c r="C144" t="s">
+        <v>132</v>
+      </c>
+      <c r="D144" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
+        <v>150</v>
+      </c>
+      <c r="B145" t="s">
+        <v>11</v>
+      </c>
+      <c r="C145" t="s">
+        <v>151</v>
+      </c>
+      <c r="D145" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>150</v>
+      </c>
+      <c r="B146" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" t="s">
+        <v>151</v>
+      </c>
+      <c r="D146" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
+        <v>150</v>
+      </c>
+      <c r="B147" t="s">
+        <v>6</v>
+      </c>
+      <c r="C147" t="s">
+        <v>151</v>
+      </c>
+      <c r="D147" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
+        <v>150</v>
+      </c>
+      <c r="B148" t="s">
+        <v>14</v>
+      </c>
+      <c r="C148" t="s">
+        <v>151</v>
+      </c>
+      <c r="D148" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
+        <v>150</v>
+      </c>
+      <c r="B149" t="s">
+        <v>16</v>
+      </c>
+      <c r="C149" t="s">
+        <v>151</v>
+      </c>
+      <c r="D149" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>150</v>
+      </c>
+      <c r="B150" t="s">
+        <v>9</v>
+      </c>
+      <c r="C150" t="s">
+        <v>151</v>
+      </c>
+      <c r="D150" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
+        <v>152</v>
+      </c>
+      <c r="B151" t="s">
+        <v>11</v>
+      </c>
+      <c r="C151" t="s">
+        <v>153</v>
+      </c>
+      <c r="D151" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>152</v>
+      </c>
+      <c r="B152" t="s">
+        <v>7</v>
+      </c>
+      <c r="C152" t="s">
+        <v>153</v>
+      </c>
+      <c r="D152" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>6</v>
+      </c>
+      <c r="C153" t="s">
+        <v>153</v>
+      </c>
+      <c r="D153" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
+        <v>152</v>
+      </c>
+      <c r="B154" t="s">
+        <v>14</v>
+      </c>
+      <c r="C154" t="s">
+        <v>153</v>
+      </c>
+      <c r="D154" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
+        <v>152</v>
+      </c>
+      <c r="B155" t="s">
+        <v>16</v>
+      </c>
+      <c r="C155" t="s">
+        <v>153</v>
+      </c>
+      <c r="D155" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>152</v>
+      </c>
+      <c r="B156" t="s">
+        <v>9</v>
+      </c>
+      <c r="C156" t="s">
+        <v>153</v>
+      </c>
+      <c r="D156" t="s">
+        <v>153</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E137" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E156" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>